<commit_message>
adding Timepix readout enable/disable commands
</commit_message>
<xml_diff>
--- a/commands/timepix/timepix_command_deck.xlsx
+++ b/commands/timepix/timepix_command_deck.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thanasi/Documents/FOXSI/Data/formatter/foxsi-4matter/foxsi4-commands/commands/timepix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B09BCDE-3EF5-5B48-8ED8-BE4572EF0348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96EFF819-8F24-5942-BFD0-789C8EEFBE3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17880" xr2:uid="{1DE950B2-129E-5A4D-8896-FB78BBCF4CAC}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17840" xr2:uid="{1DE950B2-129E-5A4D-8896-FB78BBCF4CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="all_systems" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="94">
   <si>
     <t>R=1/W=0</t>
   </si>
@@ -304,6 +304,18 @@
   </si>
   <si>
     <t>read photon data for most recent 360 events</t>
+  </si>
+  <si>
+    <t>readout_disable</t>
+  </si>
+  <si>
+    <t>readout_enable</t>
+  </si>
+  <si>
+    <t>disable telemetry readout from Timepix to Formatter</t>
+  </si>
+  <si>
+    <t>enable telemetry readout from Timepix to Formatter</t>
   </si>
 </sst>
 </file>
@@ -488,9 +500,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -528,7 +540,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -634,7 +646,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -776,7 +788,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -784,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{283F008E-2DBD-E446-BC2F-AA0D9FF4122A}">
-  <dimension ref="A1:AE22"/>
+  <dimension ref="A1:AE24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
@@ -1030,7 +1042,7 @@
         <v>0x80</v>
       </c>
       <c r="AB3" s="26">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AC3" s="26" t="s">
         <v>82</v>
@@ -1127,7 +1139,7 @@
         <v>0x88</v>
       </c>
       <c r="AB4" s="26">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AC4" s="26" t="s">
         <v>82</v>
@@ -1224,7 +1236,7 @@
         <v>0x89</v>
       </c>
       <c r="AB5" s="26">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AC5" s="26" t="s">
         <v>82</v>
@@ -1321,7 +1333,7 @@
         <v>0x8A</v>
       </c>
       <c r="AB6" s="26">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AC6" s="26" t="s">
         <v>82</v>
@@ -1418,7 +1430,7 @@
         <v>0x8B</v>
       </c>
       <c r="AB7" s="26">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AC7" s="26" t="s">
         <v>82</v>
@@ -1515,7 +1527,7 @@
         <v>0xA4</v>
       </c>
       <c r="AB8" s="26">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AC8" s="26" t="s">
         <v>82</v>
@@ -1612,7 +1624,7 @@
         <v>0xA5</v>
       </c>
       <c r="AB9" s="26">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AC9" s="26" t="s">
         <v>82</v>
@@ -1709,7 +1721,7 @@
         <v>0xA0</v>
       </c>
       <c r="AB10" s="26">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AC10" s="26" t="s">
         <v>82</v>
@@ -1806,7 +1818,7 @@
         <v>0x81</v>
       </c>
       <c r="AB11" s="26">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AC11" s="26" t="s">
         <v>82</v>
@@ -1929,11 +1941,11 @@
         <v>29</v>
       </c>
       <c r="AA13" s="25" t="str">
-        <f t="shared" ref="AA13:AA22" si="3">$E13</f>
+        <f t="shared" ref="AA13:AA24" si="3">$E13</f>
         <v>0x62</v>
       </c>
       <c r="AB13" s="26">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC13" s="26" t="s">
         <v>82</v>
@@ -2030,7 +2042,7 @@
         <v>0x63</v>
       </c>
       <c r="AB14" s="26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC14" s="26" t="s">
         <v>82</v>
@@ -2127,7 +2139,7 @@
         <v>0x22</v>
       </c>
       <c r="AB15" s="26">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AC15" s="26" t="s">
         <v>83</v>
@@ -2224,7 +2236,7 @@
         <v>0x79</v>
       </c>
       <c r="AB16" s="26">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AC16" s="26" t="s">
         <v>82</v>
@@ -2321,7 +2333,7 @@
         <v>0x70</v>
       </c>
       <c r="AB17" s="26">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AC17" s="26" t="s">
         <v>82</v>
@@ -2418,7 +2430,7 @@
         <v>0x71</v>
       </c>
       <c r="AB18" s="26">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AC18" s="26" t="s">
         <v>82</v>
@@ -2515,7 +2527,7 @@
         <v>0x72</v>
       </c>
       <c r="AB19" s="26">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="AC19" s="26" t="s">
         <v>82</v>
@@ -2612,7 +2624,7 @@
         <v>0x73</v>
       </c>
       <c r="AB20" s="26">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="AC20" s="26" t="s">
         <v>82</v>
@@ -2638,7 +2650,7 @@
         <v>1110100</v>
       </c>
       <c r="E21" s="3" t="str">
-        <f t="shared" ref="E21:E22" si="4">_xlfn.CONCAT("0x", DEC2HEX(_xlfn.BITLSHIFT($C21,7) + BIN2DEC($D21)))</f>
+        <f t="shared" ref="E21:E24" si="4">_xlfn.CONCAT("0x", DEC2HEX(_xlfn.BITLSHIFT($C21,7) + BIN2DEC($D21)))</f>
         <v>0x74</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -2709,7 +2721,7 @@
         <v>0x74</v>
       </c>
       <c r="AB21" s="26">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AC21" s="26" t="s">
         <v>82</v>
@@ -2806,7 +2818,7 @@
         <v>0x78</v>
       </c>
       <c r="AB22" s="26">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="AC22" s="26" t="s">
         <v>82</v>
@@ -2816,6 +2828,200 @@
       </c>
       <c r="AE22" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
+      </c>
+      <c r="D23" s="10">
+        <v>110000</v>
+      </c>
+      <c r="E23" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>0x30</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="L23" s="6">
+        <v>0</v>
+      </c>
+      <c r="M23" s="6">
+        <v>0</v>
+      </c>
+      <c r="N23" s="6">
+        <v>0</v>
+      </c>
+      <c r="O23" s="6">
+        <v>0</v>
+      </c>
+      <c r="P23" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>0</v>
+      </c>
+      <c r="R23" s="6">
+        <v>0</v>
+      </c>
+      <c r="S23" s="6">
+        <v>0</v>
+      </c>
+      <c r="T23" s="6">
+        <v>0</v>
+      </c>
+      <c r="U23" s="6">
+        <v>0</v>
+      </c>
+      <c r="V23" s="6">
+        <v>0</v>
+      </c>
+      <c r="W23" s="16">
+        <v>1</v>
+      </c>
+      <c r="X23" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y23" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA23" s="25" t="str">
+        <f t="shared" si="3"/>
+        <v>0x30</v>
+      </c>
+      <c r="AB23" s="26">
+        <v>2</v>
+      </c>
+      <c r="AC23" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="24" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0</v>
+      </c>
+      <c r="D24" s="10">
+        <v>110001</v>
+      </c>
+      <c r="E24" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>0x31</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="L24" s="6">
+        <v>0</v>
+      </c>
+      <c r="M24" s="6">
+        <v>0</v>
+      </c>
+      <c r="N24" s="6">
+        <v>0</v>
+      </c>
+      <c r="O24" s="6">
+        <v>0</v>
+      </c>
+      <c r="P24" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="6">
+        <v>0</v>
+      </c>
+      <c r="S24" s="6">
+        <v>0</v>
+      </c>
+      <c r="T24" s="6">
+        <v>0</v>
+      </c>
+      <c r="U24" s="6">
+        <v>0</v>
+      </c>
+      <c r="V24" s="6">
+        <v>0</v>
+      </c>
+      <c r="W24" s="16">
+        <v>1</v>
+      </c>
+      <c r="X24" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y24" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z24" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA24" s="25" t="str">
+        <f t="shared" si="3"/>
+        <v>0x31</v>
+      </c>
+      <c r="AB24" s="26">
+        <v>1</v>
+      </c>
+      <c r="AC24" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>